<commit_message>
Add Sprint 4 documentation updates
</commit_message>
<xml_diff>
--- a/documentation/scrum/Sprint_1_Burndown_Chart.xlsx
+++ b/documentation/scrum/Sprint_1_Burndown_Chart.xlsx
@@ -8,18 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://micloud365-my.sharepoint.com/personal/imashai_millenniumitesp_com/Documents/Desktop/MSc BInA/Academics/3-Interactive Visualization/Assesment/Project/group4-interactive-visualisation/documentation/scrum/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="122" documentId="11_2C750128247682E81B996B25C37309B4575122DD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61AECF1C-F1B8-4178-8CEE-61A0AFC791A8}"/>
+  <xr:revisionPtr revIDLastSave="124" documentId="11_2C750128247682E81B996B25C37309B4575122DD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{043D8B29-3842-4146-9703-991A40BF1701}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="380" windowWidth="19200" windowHeight="11280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint 1 Burndown" sheetId="1" r:id="rId1"/>
     <sheet name="Task Register" sheetId="2" r:id="rId2"/>
     <sheet name="Instructions" sheetId="3" r:id="rId3"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId4"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Task Register'!$A$1:$F$21</definedName>
   </definedNames>
@@ -112,9 +109,6 @@
     <t>To Do</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>S1-02</t>
   </si>
   <si>
@@ -335,6 +329,9 @@
   </si>
   <si>
     <t>Day 0 (20 Sep 2026) is the Sprint 1 kickoff, when all 20 checklist items (S1-01 to S1-20) were open. Five planning items were closed on Day 0 per the actual Trello count (S1-01 to S1-05: review assessment requirements, select project topic, select dataset, identify target audience, define overarching research question), leaving 15 items open at the end of Day 0.</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -811,110 +808,8 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Sprint 2 Burndown"/>
-      <sheetName val="Task Register"/>
-      <sheetName val="Instructions"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="1">
-          <cell r="C1" t="str">
-            <v>Planned Remaining</v>
-          </cell>
-          <cell r="D1" t="str">
-            <v>Actual Remaining</v>
-          </cell>
-        </row>
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>Day 0</v>
-          </cell>
-          <cell r="C2">
-            <v>19</v>
-          </cell>
-          <cell r="D2">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>Day 1</v>
-          </cell>
-          <cell r="C3">
-            <v>16</v>
-          </cell>
-          <cell r="D3">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>Day 2</v>
-          </cell>
-          <cell r="C4">
-            <v>13</v>
-          </cell>
-          <cell r="D4">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>Day 3</v>
-          </cell>
-          <cell r="C5">
-            <v>10</v>
-          </cell>
-          <cell r="D5">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>Day 4</v>
-          </cell>
-          <cell r="C6">
-            <v>6</v>
-          </cell>
-          <cell r="D6">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>Day 5</v>
-          </cell>
-          <cell r="C7">
-            <v>3</v>
-          </cell>
-          <cell r="D7">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>Day 6</v>
-          </cell>
-          <cell r="C8">
-            <v>0</v>
-          </cell>
-          <cell r="D8">
-            <v>0</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1250,7 +1145,7 @@
         <v>5</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -1270,7 +1165,7 @@
         <v>3</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -1291,7 +1186,7 @@
         <v>3</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -1312,7 +1207,7 @@
         <v>2</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -1333,7 +1228,7 @@
         <v>3</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -1354,12 +1249,12 @@
         <v>2</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B8" s="4">
         <v>46291</v>
@@ -1375,7 +1270,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
@@ -1430,10 +1325,10 @@
         <v>17</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
@@ -1453,10 +1348,10 @@
         <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -1464,13 +1359,13 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
         <v>21</v>
@@ -1479,10 +1374,10 @@
         <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -1490,13 +1385,13 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
         <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D4" t="s">
         <v>21</v>
@@ -1505,10 +1400,10 @@
         <v>22</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -1516,25 +1411,25 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
       </c>
       <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
         <v>29</v>
-      </c>
-      <c r="D5" t="s">
-        <v>30</v>
       </c>
       <c r="E5" t="s">
         <v>22</v>
       </c>
       <c r="F5" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -1542,13 +1437,13 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D6" t="s">
         <v>21</v>
@@ -1557,10 +1452,10 @@
         <v>22</v>
       </c>
       <c r="F6" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -1568,13 +1463,13 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
         <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D7" t="s">
         <v>21</v>
@@ -1583,10 +1478,10 @@
         <v>22</v>
       </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -1594,13 +1489,13 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
         <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s">
         <v>21</v>
@@ -1609,10 +1504,10 @@
         <v>22</v>
       </c>
       <c r="F8" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -1620,13 +1515,13 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B9" t="s">
         <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
         <v>21</v>
@@ -1635,10 +1530,10 @@
         <v>22</v>
       </c>
       <c r="F9" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -1646,13 +1541,13 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" t="s">
         <v>39</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>40</v>
-      </c>
-      <c r="C10" t="s">
-        <v>41</v>
       </c>
       <c r="D10" t="s">
         <v>21</v>
@@ -1661,10 +1556,10 @@
         <v>22</v>
       </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H10">
         <v>2</v>
@@ -1672,13 +1567,13 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" t="s">
         <v>42</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>43</v>
       </c>
       <c r="D11" t="s">
         <v>21</v>
@@ -1687,10 +1582,10 @@
         <v>22</v>
       </c>
       <c r="F11" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H11">
         <v>2</v>
@@ -1698,13 +1593,13 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" t="s">
         <v>44</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>45</v>
       </c>
       <c r="D12" t="s">
         <v>21</v>
@@ -1713,10 +1608,10 @@
         <v>22</v>
       </c>
       <c r="F12" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H12">
         <v>2</v>
@@ -1724,13 +1619,13 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" t="s">
         <v>46</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>47</v>
-      </c>
-      <c r="C13" t="s">
-        <v>48</v>
       </c>
       <c r="D13" t="s">
         <v>21</v>
@@ -1739,10 +1634,10 @@
         <v>22</v>
       </c>
       <c r="F13" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H13">
         <v>3</v>
@@ -1750,25 +1645,25 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" t="s">
         <v>49</v>
       </c>
-      <c r="B14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C14" t="s">
-        <v>50</v>
-      </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E14" t="s">
         <v>22</v>
       </c>
       <c r="F14" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H14">
         <v>3</v>
@@ -1776,13 +1671,13 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" t="s">
         <v>51</v>
-      </c>
-      <c r="B15" t="s">
-        <v>47</v>
-      </c>
-      <c r="C15" t="s">
-        <v>52</v>
       </c>
       <c r="D15" t="s">
         <v>21</v>
@@ -1791,10 +1686,10 @@
         <v>22</v>
       </c>
       <c r="F15" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H15">
         <v>4</v>
@@ -1802,25 +1697,25 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" t="s">
         <v>53</v>
       </c>
-      <c r="B16" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" t="s">
-        <v>54</v>
-      </c>
       <c r="D16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E16" t="s">
         <v>22</v>
       </c>
       <c r="F16" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H16">
         <v>4</v>
@@ -1828,25 +1723,25 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" t="s">
         <v>55</v>
       </c>
-      <c r="B17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C17" t="s">
-        <v>56</v>
-      </c>
       <c r="D17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E17" t="s">
         <v>22</v>
       </c>
       <c r="F17" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G17" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H17">
         <v>4</v>
@@ -1854,13 +1749,13 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" t="s">
         <v>57</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>58</v>
-      </c>
-      <c r="C18" t="s">
-        <v>59</v>
       </c>
       <c r="D18" t="s">
         <v>21</v>
@@ -1869,10 +1764,10 @@
         <v>22</v>
       </c>
       <c r="F18" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H18">
         <v>5</v>
@@ -1880,13 +1775,13 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" t="s">
         <v>60</v>
-      </c>
-      <c r="B19" t="s">
-        <v>58</v>
-      </c>
-      <c r="C19" t="s">
-        <v>61</v>
       </c>
       <c r="D19" t="s">
         <v>21</v>
@@ -1895,10 +1790,10 @@
         <v>22</v>
       </c>
       <c r="F19" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H19">
         <v>5</v>
@@ -1906,25 +1801,25 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" t="s">
         <v>62</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>63</v>
       </c>
-      <c r="C20" t="s">
-        <v>64</v>
-      </c>
       <c r="D20" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E20" t="s">
         <v>22</v>
       </c>
       <c r="F20" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H20">
         <v>6</v>
@@ -1932,25 +1827,25 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" t="s">
         <v>65</v>
       </c>
-      <c r="B21" t="s">
-        <v>63</v>
-      </c>
-      <c r="C21" t="s">
-        <v>66</v>
-      </c>
       <c r="D21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E21" t="s">
         <v>22</v>
       </c>
       <c r="F21" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H21">
         <v>6</v>
@@ -1973,42 +1868,42 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>96</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -2016,31 +1911,31 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Sprint 5 scrum documentation
</commit_message>
<xml_diff>
--- a/documentation/scrum/Sprint_1_Burndown_Chart.xlsx
+++ b/documentation/scrum/Sprint_1_Burndown_Chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://micloud365-my.sharepoint.com/personal/imashai_millenniumitesp_com/Documents/Desktop/MSc BInA/Academics/3-Interactive Visualization/Assesment/Project/group4-interactive-visualisation/documentation/scrum/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="124" documentId="11_2C750128247682E81B996B25C37309B4575122DD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{043D8B29-3842-4146-9703-991A40BF1701}"/>
+  <xr:revisionPtr revIDLastSave="126" documentId="11_2C750128247682E81B996B25C37309B4575122DD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D47A1D3-C78E-49E7-A697-C95D706B30D1}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="380" windowWidth="19200" windowHeight="11280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint 1 Burndown" sheetId="1" r:id="rId1"/>
@@ -1859,7 +1859,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1938,6 +1938,9 @@
         <v>80</v>
       </c>
     </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="6"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>